<commit_message>
Pantallas más claras, borrar todos los datos e importación que no mezcla medicamentos
- Detalle del medicamento: la barra muestra la existencia y el punto de
  reorden con sus números, «Pedir en» entre las cifras y mensajes que
  nombran el punto de reorden. Se quita la sección «Cálculo del inventario».
- Inventario: columnas «Pedir al llegar a» y «Cuánto pedir».
- Despacho: la existencia se muestra con su unidad.
- «Sin ventas en la ventana» pasa a «Sin despachos en la ventana».
- Configuración: «Borrar todos los datos» (hay que escribir BORRAR);
  conserva la configuración y las simulaciones.
- Importación: el código solo identifica un medicamento si también
  coincide el nombre, y dos filas no pueden actualizar el mismo.
- Excel de ejemplo sin «Stock seguridad» ni «Punto reorden»: los calcula
  el programa.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/datos/ejemplo_migracion_desde_excel.xlsx
+++ b/datos/ejemplo_migracion_desde_excel.xlsx
@@ -446,7 +446,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M13"/>
+  <dimension ref="A1:K13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -460,8 +460,6 @@
     <col width="11" customWidth="1" min="9" max="9"/>
     <col width="7" customWidth="1" min="10" max="10"/>
     <col width="12" customWidth="1" min="11" max="11"/>
-    <col width="10" customWidth="1" min="12" max="12"/>
-    <col width="10" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -520,16 +518,6 @@
           <t>Vencimiento</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
-        <is>
-          <t>Stock seguridad</t>
-        </is>
-      </c>
-      <c r="M1" s="1" t="inlineStr">
-        <is>
-          <t>Punto reorden</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -577,12 +565,6 @@
       <c r="K2" s="4" t="n">
         <v>46630</v>
       </c>
-      <c r="L2" s="2" t="n">
-        <v>18</v>
-      </c>
-      <c r="M2" s="2" t="n">
-        <v>42</v>
-      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -630,12 +612,6 @@
       <c r="K3" s="4" t="n">
         <v>46538</v>
       </c>
-      <c r="L3" s="2" t="n">
-        <v>33</v>
-      </c>
-      <c r="M3" s="2" t="n">
-        <v>77</v>
-      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -683,12 +659,6 @@
       <c r="K4" s="4" t="n">
         <v>46477</v>
       </c>
-      <c r="L4" s="2" t="n">
-        <v>24</v>
-      </c>
-      <c r="M4" s="2" t="n">
-        <v>56</v>
-      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -736,12 +706,6 @@
       <c r="K5" s="4" t="n">
         <v>46418</v>
       </c>
-      <c r="L5" s="2" t="n">
-        <v>9</v>
-      </c>
-      <c r="M5" s="2" t="n">
-        <v>21</v>
-      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -789,12 +753,6 @@
       <c r="K6" s="4" t="n">
         <v>46568</v>
       </c>
-      <c r="L6" s="2" t="n">
-        <v>15</v>
-      </c>
-      <c r="M6" s="2" t="n">
-        <v>35</v>
-      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -842,12 +800,6 @@
       <c r="K7" s="4" t="n">
         <v>46660</v>
       </c>
-      <c r="L7" s="2" t="n">
-        <v>12</v>
-      </c>
-      <c r="M7" s="2" t="n">
-        <v>28</v>
-      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -895,12 +847,6 @@
       <c r="K8" s="4" t="n">
         <v>46507</v>
       </c>
-      <c r="L8" s="2" t="n">
-        <v>15</v>
-      </c>
-      <c r="M8" s="2" t="n">
-        <v>35</v>
-      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -948,12 +894,6 @@
       <c r="K9" s="4" t="n">
         <v>46812</v>
       </c>
-      <c r="L9" s="2" t="n">
-        <v>27</v>
-      </c>
-      <c r="M9" s="2" t="n">
-        <v>63</v>
-      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -1001,12 +941,6 @@
       <c r="K10" s="4" t="n">
         <v>46783</v>
       </c>
-      <c r="L10" s="2" t="n">
-        <v>30</v>
-      </c>
-      <c r="M10" s="2" t="n">
-        <v>70</v>
-      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -1054,12 +988,6 @@
       <c r="K11" s="4" t="n">
         <v>46599</v>
       </c>
-      <c r="L11" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="M11" s="2" t="n">
-        <v>18</v>
-      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -1107,12 +1035,6 @@
       <c r="K12" s="4" t="n">
         <v>46721</v>
       </c>
-      <c r="L12" s="2" t="n">
-        <v>12</v>
-      </c>
-      <c r="M12" s="2" t="n">
-        <v>28</v>
-      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -1159,12 +1081,6 @@
       </c>
       <c r="K13" s="4" t="n">
         <v>46446</v>
-      </c>
-      <c r="L13" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="M13" s="2" t="n">
-        <v>6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>